<commit_message>
Semana # 7 clase # 2
</commit_message>
<xml_diff>
--- a/data/output/reporte_clientes_cerrados.xlsx
+++ b/data/output/reporte_clientes_cerrados.xlsx
@@ -443,7 +443,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>fecha_cierre</t>
+          <t>valor_contrato</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -454,11 +454,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Acme Corp</t>
+          <t>Theta SA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -471,11 +471,11 @@
           <t>Tecnología</t>
         </is>
       </c>
-      <c r="E2" s="1" t="n">
-        <v>45366</v>
+      <c r="E2" t="n">
+        <v>12000</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>45366</v>
+        <v>45387</v>
       </c>
     </row>
     <row r="3">
@@ -497,8 +497,8 @@
           <t>Manufactura</t>
         </is>
       </c>
-      <c r="E3" s="1" t="n">
-        <v>45350</v>
+      <c r="E3" t="n">
+        <v>8100</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>45350</v>
@@ -506,11 +506,11 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Eta Inc</t>
+          <t>Mu Inc</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -523,20 +523,20 @@
           <t>Manufactura</t>
         </is>
       </c>
-      <c r="E4" s="1" t="n">
-        <v>45301</v>
+      <c r="E4" t="n">
+        <v>7800</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>45301</v>
+        <v>45373</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Theta SA</t>
+          <t>Acme Corp</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -549,63 +549,63 @@
           <t>Tecnología</t>
         </is>
       </c>
-      <c r="E5" s="1" t="n">
-        <v>45387</v>
+      <c r="E5" t="n">
+        <v>4500</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>45387</v>
+        <v>45366</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mu Inc</t>
+          <t>Xi Ltd</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Manufactura</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>45373</v>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>4100</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>45373</v>
+        <v>45336</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Xi Ltd</t>
+          <t>Eta Inc</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>45336</v>
+          <t>Manufactura</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>3300</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>45336</v>
+        <v>45301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>